<commit_message>
Updated schedule, created class for : player, camera and obstacle
</commit_message>
<xml_diff>
--- a/Doc/GANTT.xlsx
+++ b/Doc/GANTT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\Cours\3eme\Atelier\PRE-TPI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leones1\Desktop\DIMEN\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBD6AC5B-BBE9-4D49-81F6-49057EF3EA3F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58F7A27-086D-4786-BEAF-CF3192B0030A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{82196E9E-969C-41C4-8C76-6F835B01D2A9}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{82196E9E-969C-41C4-8C76-6F835B01D2A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="5" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="46">
   <si>
     <t>Semaine 1</t>
   </si>
@@ -161,6 +161,9 @@
   </si>
   <si>
     <t>Documentation et finalisation (env. 36 périodes)</t>
+  </si>
+  <si>
+    <t>Création du menu de démarrage (2 périodes)</t>
   </si>
 </sst>
 </file>
@@ -515,7 +518,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -563,20 +566,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="3" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="3" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="3" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -601,12 +593,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Insatisfaisant" xfId="2" builtinId="27"/>
@@ -939,10 +945,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:147" ht="33" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="49"/>
+      <c r="B1" s="45"/>
       <c r="DY1" s="3"/>
       <c r="DZ1" s="3"/>
       <c r="EA1" s="3"/>
@@ -964,154 +970,154 @@
       <c r="EQ1" s="3"/>
     </row>
     <row r="2" spans="1:147" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="41" t="s">
+      <c r="B2" s="46"/>
+      <c r="C2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="42"/>
-      <c r="O2" s="42"/>
-      <c r="P2" s="42"/>
-      <c r="Q2" s="41" t="s">
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="42"/>
-      <c r="S2" s="42"/>
-      <c r="T2" s="42"/>
-      <c r="U2" s="42"/>
-      <c r="V2" s="42"/>
-      <c r="W2" s="42"/>
-      <c r="X2" s="42"/>
-      <c r="Y2" s="42"/>
-      <c r="Z2" s="42"/>
-      <c r="AA2" s="42"/>
-      <c r="AB2" s="42"/>
-      <c r="AC2" s="42"/>
-      <c r="AD2" s="42"/>
-      <c r="AE2" s="41" t="s">
+      <c r="R2" s="37"/>
+      <c r="S2" s="37"/>
+      <c r="T2" s="37"/>
+      <c r="U2" s="37"/>
+      <c r="V2" s="37"/>
+      <c r="W2" s="37"/>
+      <c r="X2" s="37"/>
+      <c r="Y2" s="37"/>
+      <c r="Z2" s="37"/>
+      <c r="AA2" s="37"/>
+      <c r="AB2" s="37"/>
+      <c r="AC2" s="37"/>
+      <c r="AD2" s="37"/>
+      <c r="AE2" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="AF2" s="42"/>
-      <c r="AG2" s="42"/>
-      <c r="AH2" s="42"/>
-      <c r="AI2" s="42"/>
-      <c r="AJ2" s="42"/>
-      <c r="AK2" s="42"/>
-      <c r="AL2" s="42"/>
-      <c r="AM2" s="42"/>
-      <c r="AN2" s="42"/>
-      <c r="AO2" s="42"/>
-      <c r="AP2" s="42"/>
-      <c r="AQ2" s="42"/>
-      <c r="AR2" s="42"/>
-      <c r="AS2" s="41" t="s">
+      <c r="AF2" s="37"/>
+      <c r="AG2" s="37"/>
+      <c r="AH2" s="37"/>
+      <c r="AI2" s="37"/>
+      <c r="AJ2" s="37"/>
+      <c r="AK2" s="37"/>
+      <c r="AL2" s="37"/>
+      <c r="AM2" s="37"/>
+      <c r="AN2" s="37"/>
+      <c r="AO2" s="37"/>
+      <c r="AP2" s="37"/>
+      <c r="AQ2" s="37"/>
+      <c r="AR2" s="37"/>
+      <c r="AS2" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="AT2" s="42"/>
-      <c r="AU2" s="42"/>
-      <c r="AV2" s="42"/>
-      <c r="AW2" s="42"/>
-      <c r="AX2" s="42"/>
-      <c r="AY2" s="42"/>
-      <c r="AZ2" s="42"/>
-      <c r="BA2" s="42"/>
-      <c r="BB2" s="42"/>
-      <c r="BC2" s="42"/>
-      <c r="BD2" s="42"/>
-      <c r="BE2" s="42"/>
-      <c r="BF2" s="42"/>
-      <c r="BG2" s="41" t="s">
+      <c r="AT2" s="37"/>
+      <c r="AU2" s="37"/>
+      <c r="AV2" s="37"/>
+      <c r="AW2" s="37"/>
+      <c r="AX2" s="37"/>
+      <c r="AY2" s="37"/>
+      <c r="AZ2" s="37"/>
+      <c r="BA2" s="37"/>
+      <c r="BB2" s="37"/>
+      <c r="BC2" s="37"/>
+      <c r="BD2" s="37"/>
+      <c r="BE2" s="37"/>
+      <c r="BF2" s="37"/>
+      <c r="BG2" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="BH2" s="42"/>
-      <c r="BI2" s="42"/>
-      <c r="BJ2" s="42"/>
-      <c r="BK2" s="42"/>
-      <c r="BL2" s="42"/>
-      <c r="BM2" s="42"/>
-      <c r="BN2" s="42"/>
-      <c r="BO2" s="42"/>
-      <c r="BP2" s="42"/>
-      <c r="BQ2" s="42"/>
-      <c r="BR2" s="42"/>
-      <c r="BS2" s="42"/>
-      <c r="BT2" s="42"/>
-      <c r="BU2" s="41" t="s">
+      <c r="BH2" s="37"/>
+      <c r="BI2" s="37"/>
+      <c r="BJ2" s="37"/>
+      <c r="BK2" s="37"/>
+      <c r="BL2" s="37"/>
+      <c r="BM2" s="37"/>
+      <c r="BN2" s="37"/>
+      <c r="BO2" s="37"/>
+      <c r="BP2" s="37"/>
+      <c r="BQ2" s="37"/>
+      <c r="BR2" s="37"/>
+      <c r="BS2" s="37"/>
+      <c r="BT2" s="37"/>
+      <c r="BU2" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="BV2" s="42"/>
-      <c r="BW2" s="42"/>
-      <c r="BX2" s="42"/>
-      <c r="BY2" s="42"/>
-      <c r="BZ2" s="42"/>
-      <c r="CA2" s="42"/>
-      <c r="CB2" s="42"/>
-      <c r="CC2" s="42"/>
-      <c r="CD2" s="42"/>
-      <c r="CE2" s="42"/>
-      <c r="CF2" s="42"/>
-      <c r="CG2" s="42"/>
-      <c r="CH2" s="42"/>
-      <c r="CI2" s="41" t="s">
+      <c r="BV2" s="37"/>
+      <c r="BW2" s="37"/>
+      <c r="BX2" s="37"/>
+      <c r="BY2" s="37"/>
+      <c r="BZ2" s="37"/>
+      <c r="CA2" s="37"/>
+      <c r="CB2" s="37"/>
+      <c r="CC2" s="37"/>
+      <c r="CD2" s="37"/>
+      <c r="CE2" s="37"/>
+      <c r="CF2" s="37"/>
+      <c r="CG2" s="37"/>
+      <c r="CH2" s="37"/>
+      <c r="CI2" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="CJ2" s="42"/>
-      <c r="CK2" s="42"/>
-      <c r="CL2" s="42"/>
-      <c r="CM2" s="42"/>
-      <c r="CN2" s="42"/>
-      <c r="CO2" s="42"/>
-      <c r="CP2" s="42"/>
-      <c r="CQ2" s="42"/>
-      <c r="CR2" s="42"/>
-      <c r="CS2" s="42"/>
-      <c r="CT2" s="42"/>
-      <c r="CU2" s="42"/>
-      <c r="CV2" s="42"/>
-      <c r="CW2" s="41" t="s">
+      <c r="CJ2" s="37"/>
+      <c r="CK2" s="37"/>
+      <c r="CL2" s="37"/>
+      <c r="CM2" s="37"/>
+      <c r="CN2" s="37"/>
+      <c r="CO2" s="37"/>
+      <c r="CP2" s="37"/>
+      <c r="CQ2" s="37"/>
+      <c r="CR2" s="37"/>
+      <c r="CS2" s="37"/>
+      <c r="CT2" s="37"/>
+      <c r="CU2" s="37"/>
+      <c r="CV2" s="37"/>
+      <c r="CW2" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="CX2" s="42"/>
-      <c r="CY2" s="42"/>
-      <c r="CZ2" s="42"/>
-      <c r="DA2" s="42"/>
-      <c r="DB2" s="42"/>
-      <c r="DC2" s="42"/>
-      <c r="DD2" s="42"/>
-      <c r="DE2" s="42"/>
-      <c r="DF2" s="42"/>
-      <c r="DG2" s="42"/>
-      <c r="DH2" s="42"/>
-      <c r="DI2" s="42"/>
-      <c r="DJ2" s="42"/>
-      <c r="DK2" s="47" t="s">
+      <c r="CX2" s="37"/>
+      <c r="CY2" s="37"/>
+      <c r="CZ2" s="37"/>
+      <c r="DA2" s="37"/>
+      <c r="DB2" s="37"/>
+      <c r="DC2" s="37"/>
+      <c r="DD2" s="37"/>
+      <c r="DE2" s="37"/>
+      <c r="DF2" s="37"/>
+      <c r="DG2" s="37"/>
+      <c r="DH2" s="37"/>
+      <c r="DI2" s="37"/>
+      <c r="DJ2" s="37"/>
+      <c r="DK2" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="DL2" s="47"/>
-      <c r="DM2" s="47"/>
-      <c r="DN2" s="47"/>
-      <c r="DO2" s="47"/>
-      <c r="DP2" s="47"/>
-      <c r="DQ2" s="47"/>
-      <c r="DR2" s="47"/>
-      <c r="DS2" s="47"/>
-      <c r="DT2" s="47"/>
-      <c r="DU2" s="47"/>
-      <c r="DV2" s="47"/>
-      <c r="DW2" s="47"/>
-      <c r="DX2" s="47"/>
+      <c r="DL2" s="42"/>
+      <c r="DM2" s="42"/>
+      <c r="DN2" s="42"/>
+      <c r="DO2" s="42"/>
+      <c r="DP2" s="42"/>
+      <c r="DQ2" s="42"/>
+      <c r="DR2" s="42"/>
+      <c r="DS2" s="42"/>
+      <c r="DT2" s="42"/>
+      <c r="DU2" s="42"/>
+      <c r="DV2" s="42"/>
+      <c r="DW2" s="42"/>
+      <c r="DX2" s="42"/>
       <c r="DY2" s="3"/>
       <c r="DZ2" s="3"/>
       <c r="EA2" s="3"/>
@@ -1133,134 +1139,134 @@
       <c r="EQ2" s="3"/>
     </row>
     <row r="3" spans="1:147" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50"/>
-      <c r="B3" s="50"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="44"/>
-      <c r="Q3" s="43"/>
-      <c r="R3" s="44"/>
-      <c r="S3" s="44"/>
-      <c r="T3" s="44"/>
-      <c r="U3" s="44"/>
-      <c r="V3" s="44"/>
-      <c r="W3" s="44"/>
-      <c r="X3" s="44"/>
-      <c r="Y3" s="44"/>
-      <c r="Z3" s="44"/>
-      <c r="AA3" s="44"/>
-      <c r="AB3" s="44"/>
-      <c r="AC3" s="44"/>
-      <c r="AD3" s="44"/>
-      <c r="AE3" s="43"/>
-      <c r="AF3" s="44"/>
-      <c r="AG3" s="44"/>
-      <c r="AH3" s="44"/>
-      <c r="AI3" s="44"/>
-      <c r="AJ3" s="44"/>
-      <c r="AK3" s="44"/>
-      <c r="AL3" s="44"/>
-      <c r="AM3" s="44"/>
-      <c r="AN3" s="44"/>
-      <c r="AO3" s="44"/>
-      <c r="AP3" s="44"/>
-      <c r="AQ3" s="44"/>
-      <c r="AR3" s="44"/>
-      <c r="AS3" s="43"/>
-      <c r="AT3" s="44"/>
-      <c r="AU3" s="44"/>
-      <c r="AV3" s="44"/>
-      <c r="AW3" s="44"/>
-      <c r="AX3" s="44"/>
-      <c r="AY3" s="44"/>
-      <c r="AZ3" s="44"/>
-      <c r="BA3" s="44"/>
-      <c r="BB3" s="44"/>
-      <c r="BC3" s="44"/>
-      <c r="BD3" s="44"/>
-      <c r="BE3" s="44"/>
-      <c r="BF3" s="44"/>
-      <c r="BG3" s="43"/>
-      <c r="BH3" s="44"/>
-      <c r="BI3" s="44"/>
-      <c r="BJ3" s="44"/>
-      <c r="BK3" s="44"/>
-      <c r="BL3" s="44"/>
-      <c r="BM3" s="44"/>
-      <c r="BN3" s="44"/>
-      <c r="BO3" s="44"/>
-      <c r="BP3" s="44"/>
-      <c r="BQ3" s="44"/>
-      <c r="BR3" s="44"/>
-      <c r="BS3" s="44"/>
-      <c r="BT3" s="44"/>
-      <c r="BU3" s="43"/>
-      <c r="BV3" s="44"/>
-      <c r="BW3" s="44"/>
-      <c r="BX3" s="44"/>
-      <c r="BY3" s="44"/>
-      <c r="BZ3" s="44"/>
-      <c r="CA3" s="44"/>
-      <c r="CB3" s="44"/>
-      <c r="CC3" s="44"/>
-      <c r="CD3" s="44"/>
-      <c r="CE3" s="44"/>
-      <c r="CF3" s="44"/>
-      <c r="CG3" s="44"/>
-      <c r="CH3" s="44"/>
-      <c r="CI3" s="43"/>
-      <c r="CJ3" s="44"/>
-      <c r="CK3" s="44"/>
-      <c r="CL3" s="44"/>
-      <c r="CM3" s="44"/>
-      <c r="CN3" s="44"/>
-      <c r="CO3" s="44"/>
-      <c r="CP3" s="44"/>
-      <c r="CQ3" s="44"/>
-      <c r="CR3" s="44"/>
-      <c r="CS3" s="44"/>
-      <c r="CT3" s="44"/>
-      <c r="CU3" s="44"/>
-      <c r="CV3" s="44"/>
-      <c r="CW3" s="43"/>
-      <c r="CX3" s="44"/>
-      <c r="CY3" s="44"/>
-      <c r="CZ3" s="44"/>
-      <c r="DA3" s="44"/>
-      <c r="DB3" s="44"/>
-      <c r="DC3" s="44"/>
-      <c r="DD3" s="44"/>
-      <c r="DE3" s="44"/>
-      <c r="DF3" s="44"/>
-      <c r="DG3" s="44"/>
-      <c r="DH3" s="44"/>
-      <c r="DI3" s="44"/>
-      <c r="DJ3" s="44"/>
-      <c r="DK3" s="47"/>
-      <c r="DL3" s="47"/>
-      <c r="DM3" s="47"/>
-      <c r="DN3" s="47"/>
-      <c r="DO3" s="47"/>
-      <c r="DP3" s="47"/>
-      <c r="DQ3" s="47"/>
-      <c r="DR3" s="47"/>
-      <c r="DS3" s="47"/>
-      <c r="DT3" s="47"/>
-      <c r="DU3" s="47"/>
-      <c r="DV3" s="47"/>
-      <c r="DW3" s="47"/>
-      <c r="DX3" s="47"/>
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="38"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="39"/>
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="38"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="39"/>
+      <c r="AH3" s="39"/>
+      <c r="AI3" s="39"/>
+      <c r="AJ3" s="39"/>
+      <c r="AK3" s="39"/>
+      <c r="AL3" s="39"/>
+      <c r="AM3" s="39"/>
+      <c r="AN3" s="39"/>
+      <c r="AO3" s="39"/>
+      <c r="AP3" s="39"/>
+      <c r="AQ3" s="39"/>
+      <c r="AR3" s="39"/>
+      <c r="AS3" s="38"/>
+      <c r="AT3" s="39"/>
+      <c r="AU3" s="39"/>
+      <c r="AV3" s="39"/>
+      <c r="AW3" s="39"/>
+      <c r="AX3" s="39"/>
+      <c r="AY3" s="39"/>
+      <c r="AZ3" s="39"/>
+      <c r="BA3" s="39"/>
+      <c r="BB3" s="39"/>
+      <c r="BC3" s="39"/>
+      <c r="BD3" s="39"/>
+      <c r="BE3" s="39"/>
+      <c r="BF3" s="39"/>
+      <c r="BG3" s="38"/>
+      <c r="BH3" s="39"/>
+      <c r="BI3" s="39"/>
+      <c r="BJ3" s="39"/>
+      <c r="BK3" s="39"/>
+      <c r="BL3" s="39"/>
+      <c r="BM3" s="39"/>
+      <c r="BN3" s="39"/>
+      <c r="BO3" s="39"/>
+      <c r="BP3" s="39"/>
+      <c r="BQ3" s="39"/>
+      <c r="BR3" s="39"/>
+      <c r="BS3" s="39"/>
+      <c r="BT3" s="39"/>
+      <c r="BU3" s="38"/>
+      <c r="BV3" s="39"/>
+      <c r="BW3" s="39"/>
+      <c r="BX3" s="39"/>
+      <c r="BY3" s="39"/>
+      <c r="BZ3" s="39"/>
+      <c r="CA3" s="39"/>
+      <c r="CB3" s="39"/>
+      <c r="CC3" s="39"/>
+      <c r="CD3" s="39"/>
+      <c r="CE3" s="39"/>
+      <c r="CF3" s="39"/>
+      <c r="CG3" s="39"/>
+      <c r="CH3" s="39"/>
+      <c r="CI3" s="38"/>
+      <c r="CJ3" s="39"/>
+      <c r="CK3" s="39"/>
+      <c r="CL3" s="39"/>
+      <c r="CM3" s="39"/>
+      <c r="CN3" s="39"/>
+      <c r="CO3" s="39"/>
+      <c r="CP3" s="39"/>
+      <c r="CQ3" s="39"/>
+      <c r="CR3" s="39"/>
+      <c r="CS3" s="39"/>
+      <c r="CT3" s="39"/>
+      <c r="CU3" s="39"/>
+      <c r="CV3" s="39"/>
+      <c r="CW3" s="38"/>
+      <c r="CX3" s="39"/>
+      <c r="CY3" s="39"/>
+      <c r="CZ3" s="39"/>
+      <c r="DA3" s="39"/>
+      <c r="DB3" s="39"/>
+      <c r="DC3" s="39"/>
+      <c r="DD3" s="39"/>
+      <c r="DE3" s="39"/>
+      <c r="DF3" s="39"/>
+      <c r="DG3" s="39"/>
+      <c r="DH3" s="39"/>
+      <c r="DI3" s="39"/>
+      <c r="DJ3" s="39"/>
+      <c r="DK3" s="42"/>
+      <c r="DL3" s="42"/>
+      <c r="DM3" s="42"/>
+      <c r="DN3" s="42"/>
+      <c r="DO3" s="42"/>
+      <c r="DP3" s="42"/>
+      <c r="DQ3" s="42"/>
+      <c r="DR3" s="42"/>
+      <c r="DS3" s="42"/>
+      <c r="DT3" s="42"/>
+      <c r="DU3" s="42"/>
+      <c r="DV3" s="42"/>
+      <c r="DW3" s="42"/>
+      <c r="DX3" s="42"/>
       <c r="DY3" s="3"/>
       <c r="DZ3" s="3"/>
       <c r="EA3" s="3"/>
@@ -1282,134 +1288,134 @@
       <c r="EQ3" s="3"/>
     </row>
     <row r="4" spans="1:147" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="50"/>
-      <c r="B4" s="50"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
-      <c r="M4" s="46"/>
-      <c r="N4" s="46"/>
-      <c r="O4" s="46"/>
-      <c r="P4" s="46"/>
-      <c r="Q4" s="45"/>
-      <c r="R4" s="46"/>
-      <c r="S4" s="46"/>
-      <c r="T4" s="46"/>
-      <c r="U4" s="46"/>
-      <c r="V4" s="46"/>
-      <c r="W4" s="46"/>
-      <c r="X4" s="46"/>
-      <c r="Y4" s="46"/>
-      <c r="Z4" s="46"/>
-      <c r="AA4" s="46"/>
-      <c r="AB4" s="46"/>
-      <c r="AC4" s="46"/>
-      <c r="AD4" s="46"/>
-      <c r="AE4" s="45"/>
-      <c r="AF4" s="46"/>
-      <c r="AG4" s="46"/>
-      <c r="AH4" s="46"/>
-      <c r="AI4" s="46"/>
-      <c r="AJ4" s="46"/>
-      <c r="AK4" s="46"/>
-      <c r="AL4" s="46"/>
-      <c r="AM4" s="46"/>
-      <c r="AN4" s="46"/>
-      <c r="AO4" s="46"/>
-      <c r="AP4" s="46"/>
-      <c r="AQ4" s="46"/>
-      <c r="AR4" s="46"/>
-      <c r="AS4" s="45"/>
-      <c r="AT4" s="46"/>
-      <c r="AU4" s="46"/>
-      <c r="AV4" s="46"/>
-      <c r="AW4" s="46"/>
-      <c r="AX4" s="46"/>
-      <c r="AY4" s="46"/>
-      <c r="AZ4" s="46"/>
-      <c r="BA4" s="46"/>
-      <c r="BB4" s="46"/>
-      <c r="BC4" s="46"/>
-      <c r="BD4" s="46"/>
-      <c r="BE4" s="46"/>
-      <c r="BF4" s="46"/>
-      <c r="BG4" s="45"/>
-      <c r="BH4" s="46"/>
-      <c r="BI4" s="46"/>
-      <c r="BJ4" s="46"/>
-      <c r="BK4" s="46"/>
-      <c r="BL4" s="46"/>
-      <c r="BM4" s="46"/>
-      <c r="BN4" s="46"/>
-      <c r="BO4" s="46"/>
-      <c r="BP4" s="46"/>
-      <c r="BQ4" s="46"/>
-      <c r="BR4" s="46"/>
-      <c r="BS4" s="46"/>
-      <c r="BT4" s="46"/>
-      <c r="BU4" s="45"/>
-      <c r="BV4" s="46"/>
-      <c r="BW4" s="46"/>
-      <c r="BX4" s="46"/>
-      <c r="BY4" s="46"/>
-      <c r="BZ4" s="46"/>
-      <c r="CA4" s="46"/>
-      <c r="CB4" s="46"/>
-      <c r="CC4" s="46"/>
-      <c r="CD4" s="46"/>
-      <c r="CE4" s="46"/>
-      <c r="CF4" s="46"/>
-      <c r="CG4" s="46"/>
-      <c r="CH4" s="46"/>
-      <c r="CI4" s="45"/>
-      <c r="CJ4" s="46"/>
-      <c r="CK4" s="46"/>
-      <c r="CL4" s="46"/>
-      <c r="CM4" s="46"/>
-      <c r="CN4" s="46"/>
-      <c r="CO4" s="46"/>
-      <c r="CP4" s="46"/>
-      <c r="CQ4" s="46"/>
-      <c r="CR4" s="46"/>
-      <c r="CS4" s="46"/>
-      <c r="CT4" s="46"/>
-      <c r="CU4" s="46"/>
-      <c r="CV4" s="46"/>
-      <c r="CW4" s="45"/>
-      <c r="CX4" s="46"/>
-      <c r="CY4" s="46"/>
-      <c r="CZ4" s="46"/>
-      <c r="DA4" s="46"/>
-      <c r="DB4" s="46"/>
-      <c r="DC4" s="46"/>
-      <c r="DD4" s="46"/>
-      <c r="DE4" s="46"/>
-      <c r="DF4" s="46"/>
-      <c r="DG4" s="46"/>
-      <c r="DH4" s="46"/>
-      <c r="DI4" s="46"/>
-      <c r="DJ4" s="46"/>
-      <c r="DK4" s="47"/>
-      <c r="DL4" s="47"/>
-      <c r="DM4" s="47"/>
-      <c r="DN4" s="47"/>
-      <c r="DO4" s="47"/>
-      <c r="DP4" s="47"/>
-      <c r="DQ4" s="47"/>
-      <c r="DR4" s="47"/>
-      <c r="DS4" s="47"/>
-      <c r="DT4" s="47"/>
-      <c r="DU4" s="47"/>
-      <c r="DV4" s="47"/>
-      <c r="DW4" s="47"/>
-      <c r="DX4" s="47"/>
+      <c r="A4" s="46"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="40"/>
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="41"/>
+      <c r="V4" s="41"/>
+      <c r="W4" s="41"/>
+      <c r="X4" s="41"/>
+      <c r="Y4" s="41"/>
+      <c r="Z4" s="41"/>
+      <c r="AA4" s="41"/>
+      <c r="AB4" s="41"/>
+      <c r="AC4" s="41"/>
+      <c r="AD4" s="41"/>
+      <c r="AE4" s="40"/>
+      <c r="AF4" s="41"/>
+      <c r="AG4" s="41"/>
+      <c r="AH4" s="41"/>
+      <c r="AI4" s="41"/>
+      <c r="AJ4" s="41"/>
+      <c r="AK4" s="41"/>
+      <c r="AL4" s="41"/>
+      <c r="AM4" s="41"/>
+      <c r="AN4" s="41"/>
+      <c r="AO4" s="41"/>
+      <c r="AP4" s="41"/>
+      <c r="AQ4" s="41"/>
+      <c r="AR4" s="41"/>
+      <c r="AS4" s="40"/>
+      <c r="AT4" s="41"/>
+      <c r="AU4" s="41"/>
+      <c r="AV4" s="41"/>
+      <c r="AW4" s="41"/>
+      <c r="AX4" s="41"/>
+      <c r="AY4" s="41"/>
+      <c r="AZ4" s="41"/>
+      <c r="BA4" s="41"/>
+      <c r="BB4" s="41"/>
+      <c r="BC4" s="41"/>
+      <c r="BD4" s="41"/>
+      <c r="BE4" s="41"/>
+      <c r="BF4" s="41"/>
+      <c r="BG4" s="40"/>
+      <c r="BH4" s="41"/>
+      <c r="BI4" s="41"/>
+      <c r="BJ4" s="41"/>
+      <c r="BK4" s="41"/>
+      <c r="BL4" s="41"/>
+      <c r="BM4" s="41"/>
+      <c r="BN4" s="41"/>
+      <c r="BO4" s="41"/>
+      <c r="BP4" s="41"/>
+      <c r="BQ4" s="41"/>
+      <c r="BR4" s="41"/>
+      <c r="BS4" s="41"/>
+      <c r="BT4" s="41"/>
+      <c r="BU4" s="40"/>
+      <c r="BV4" s="41"/>
+      <c r="BW4" s="41"/>
+      <c r="BX4" s="41"/>
+      <c r="BY4" s="41"/>
+      <c r="BZ4" s="41"/>
+      <c r="CA4" s="41"/>
+      <c r="CB4" s="41"/>
+      <c r="CC4" s="41"/>
+      <c r="CD4" s="41"/>
+      <c r="CE4" s="41"/>
+      <c r="CF4" s="41"/>
+      <c r="CG4" s="41"/>
+      <c r="CH4" s="41"/>
+      <c r="CI4" s="40"/>
+      <c r="CJ4" s="41"/>
+      <c r="CK4" s="41"/>
+      <c r="CL4" s="41"/>
+      <c r="CM4" s="41"/>
+      <c r="CN4" s="41"/>
+      <c r="CO4" s="41"/>
+      <c r="CP4" s="41"/>
+      <c r="CQ4" s="41"/>
+      <c r="CR4" s="41"/>
+      <c r="CS4" s="41"/>
+      <c r="CT4" s="41"/>
+      <c r="CU4" s="41"/>
+      <c r="CV4" s="41"/>
+      <c r="CW4" s="40"/>
+      <c r="CX4" s="41"/>
+      <c r="CY4" s="41"/>
+      <c r="CZ4" s="41"/>
+      <c r="DA4" s="41"/>
+      <c r="DB4" s="41"/>
+      <c r="DC4" s="41"/>
+      <c r="DD4" s="41"/>
+      <c r="DE4" s="41"/>
+      <c r="DF4" s="41"/>
+      <c r="DG4" s="41"/>
+      <c r="DH4" s="41"/>
+      <c r="DI4" s="41"/>
+      <c r="DJ4" s="41"/>
+      <c r="DK4" s="42"/>
+      <c r="DL4" s="42"/>
+      <c r="DM4" s="42"/>
+      <c r="DN4" s="42"/>
+      <c r="DO4" s="42"/>
+      <c r="DP4" s="42"/>
+      <c r="DQ4" s="42"/>
+      <c r="DR4" s="42"/>
+      <c r="DS4" s="42"/>
+      <c r="DT4" s="42"/>
+      <c r="DU4" s="42"/>
+      <c r="DV4" s="42"/>
+      <c r="DW4" s="42"/>
+      <c r="DX4" s="42"/>
       <c r="DY4" s="3"/>
       <c r="DZ4" s="3"/>
       <c r="EA4" s="3"/>
@@ -1886,15 +1892,15 @@
       <c r="EQ7" s="3"/>
     </row>
     <row r="8" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="43" t="s">
         <v>42</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="50"/>
+      <c r="E8" s="50"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
@@ -2039,18 +2045,18 @@
       <c r="EQ8" s="3"/>
     </row>
     <row r="9" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="38"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="22" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="15"/>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
+      <c r="F9" s="50"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="50"/>
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
@@ -2190,7 +2196,7 @@
       <c r="EQ9" s="3"/>
     </row>
     <row r="10" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="38"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="24" t="s">
         <v>21</v>
       </c>
@@ -2202,10 +2208,10 @@
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
+      <c r="K10" s="50"/>
+      <c r="L10" s="50"/>
+      <c r="M10" s="50"/>
+      <c r="N10" s="50"/>
       <c r="O10" s="8"/>
       <c r="P10" s="16"/>
       <c r="Q10" s="15"/>
@@ -2341,7 +2347,7 @@
       <c r="EQ10" s="3"/>
     </row>
     <row r="11" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="38"/>
+      <c r="A11" s="44"/>
       <c r="B11" s="22" t="s">
         <v>13</v>
       </c>
@@ -2357,8 +2363,8 @@
       <c r="L11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="12"/>
+      <c r="O11" s="50"/>
+      <c r="P11" s="51"/>
       <c r="Q11" s="15"/>
       <c r="R11" s="8"/>
       <c r="S11" s="8"/>
@@ -2492,7 +2498,7 @@
       <c r="EQ11" s="3"/>
     </row>
     <row r="12" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="44" t="s">
         <v>43</v>
       </c>
       <c r="B12" s="25" t="s">
@@ -2512,12 +2518,12 @@
       <c r="N12" s="5"/>
       <c r="O12" s="5"/>
       <c r="P12" s="7"/>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="11"/>
-      <c r="S12" s="11"/>
-      <c r="T12" s="11"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="11"/>
+      <c r="Q12" s="49"/>
+      <c r="R12" s="50"/>
+      <c r="S12" s="50"/>
+      <c r="T12" s="50"/>
+      <c r="U12" s="50"/>
+      <c r="V12" s="50"/>
       <c r="W12" s="5"/>
       <c r="X12" s="5"/>
       <c r="Y12" s="5"/>
@@ -2645,7 +2651,7 @@
       <c r="EQ12" s="3"/>
     </row>
     <row r="13" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="38"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="23" t="s">
         <v>15</v>
       </c>
@@ -2669,11 +2675,11 @@
       <c r="T13" s="5"/>
       <c r="U13" s="5"/>
       <c r="V13" s="5"/>
-      <c r="W13" s="11"/>
-      <c r="X13" s="11"/>
-      <c r="Y13" s="11"/>
-      <c r="Z13" s="11"/>
-      <c r="AA13" s="11"/>
+      <c r="W13" s="50"/>
+      <c r="X13" s="50"/>
+      <c r="Y13" s="50"/>
+      <c r="Z13" s="50"/>
+      <c r="AA13" s="50"/>
       <c r="AB13" s="5"/>
       <c r="AC13" s="5"/>
       <c r="AD13" s="7"/>
@@ -2796,7 +2802,7 @@
       <c r="EQ13" s="3"/>
     </row>
     <row r="14" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="24" t="s">
         <v>16</v>
       </c>
@@ -2825,9 +2831,9 @@
       <c r="Y14" s="5"/>
       <c r="Z14" s="5"/>
       <c r="AA14" s="5"/>
-      <c r="AB14" s="11"/>
-      <c r="AC14" s="11"/>
-      <c r="AD14" s="12"/>
+      <c r="AB14" s="50"/>
+      <c r="AC14" s="50"/>
+      <c r="AD14" s="51"/>
       <c r="AE14" s="6"/>
       <c r="AF14" s="5"/>
       <c r="AG14" s="5"/>
@@ -2947,7 +2953,7 @@
       <c r="EQ14" s="3"/>
     </row>
     <row r="15" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="22" t="s">
         <v>17</v>
       </c>
@@ -2979,13 +2985,13 @@
       <c r="AB15" s="5"/>
       <c r="AC15" s="5"/>
       <c r="AD15" s="7"/>
-      <c r="AE15" s="10"/>
-      <c r="AF15" s="11"/>
-      <c r="AG15" s="11"/>
-      <c r="AH15" s="11"/>
-      <c r="AI15" s="11"/>
-      <c r="AJ15" s="11"/>
-      <c r="AK15" s="11"/>
+      <c r="AE15" s="49"/>
+      <c r="AF15" s="50"/>
+      <c r="AG15" s="50"/>
+      <c r="AH15" s="50"/>
+      <c r="AI15" s="50"/>
+      <c r="AJ15" s="50"/>
+      <c r="AK15" s="50"/>
       <c r="AL15" s="5"/>
       <c r="AM15" s="5"/>
       <c r="AN15" s="5"/>
@@ -3098,7 +3104,7 @@
       <c r="EQ15" s="3"/>
     </row>
     <row r="16" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="38"/>
+      <c r="A16" s="44"/>
       <c r="B16" s="25" t="s">
         <v>18</v>
       </c>
@@ -3137,11 +3143,11 @@
       <c r="AI16" s="5"/>
       <c r="AJ16" s="5"/>
       <c r="AK16" s="5"/>
-      <c r="AL16" s="11"/>
-      <c r="AM16" s="11"/>
-      <c r="AN16" s="11"/>
-      <c r="AO16" s="11"/>
-      <c r="AP16" s="11"/>
+      <c r="AL16" s="50"/>
+      <c r="AM16" s="50"/>
+      <c r="AN16" s="50"/>
+      <c r="AO16" s="50"/>
+      <c r="AP16" s="50"/>
       <c r="AQ16" s="5"/>
       <c r="AR16" s="7"/>
       <c r="AS16" s="6"/>
@@ -3249,7 +3255,7 @@
       <c r="EQ16" s="3"/>
     </row>
     <row r="17" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="38"/>
+      <c r="A17" s="44"/>
       <c r="B17" s="23" t="s">
         <v>22</v>
       </c>
@@ -3293,8 +3299,8 @@
       <c r="AN17" s="5"/>
       <c r="AO17" s="5"/>
       <c r="AP17" s="5"/>
-      <c r="AQ17" s="11"/>
-      <c r="AR17" s="12"/>
+      <c r="AQ17" s="50"/>
+      <c r="AR17" s="51"/>
       <c r="AS17" s="6"/>
       <c r="AT17" s="5"/>
       <c r="AU17" s="5"/>
@@ -3400,7 +3406,7 @@
       <c r="EQ17" s="3"/>
     </row>
     <row r="18" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="38"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="25" t="s">
         <v>23</v>
       </c>
@@ -3446,12 +3452,12 @@
       <c r="AP18" s="5"/>
       <c r="AQ18" s="5"/>
       <c r="AR18" s="7"/>
-      <c r="AS18" s="10"/>
-      <c r="AT18" s="11"/>
-      <c r="AU18" s="11"/>
-      <c r="AV18" s="11"/>
-      <c r="AW18" s="11"/>
-      <c r="AX18" s="11"/>
+      <c r="AS18" s="49"/>
+      <c r="AT18" s="50"/>
+      <c r="AU18" s="50"/>
+      <c r="AV18" s="50"/>
+      <c r="AW18" s="50"/>
+      <c r="AX18" s="50"/>
       <c r="AY18" s="5"/>
       <c r="AZ18" s="5"/>
       <c r="BA18" s="5"/>
@@ -3551,7 +3557,7 @@
       <c r="EQ18" s="3"/>
     </row>
     <row r="19" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="22" t="s">
         <v>24</v>
       </c>
@@ -3603,12 +3609,12 @@
       <c r="AV19" s="5"/>
       <c r="AW19" s="5"/>
       <c r="AX19" s="5"/>
-      <c r="AY19" s="11"/>
-      <c r="AZ19" s="11"/>
-      <c r="BA19" s="11"/>
-      <c r="BB19" s="11"/>
-      <c r="BC19" s="11"/>
-      <c r="BD19" s="11"/>
+      <c r="AY19" s="50"/>
+      <c r="AZ19" s="50"/>
+      <c r="BA19" s="50"/>
+      <c r="BB19" s="50"/>
+      <c r="BC19" s="50"/>
+      <c r="BD19" s="50"/>
       <c r="BE19" s="5"/>
       <c r="BF19" s="7"/>
       <c r="BG19" s="6"/>
@@ -3702,7 +3708,7 @@
       <c r="EQ19" s="3"/>
     </row>
     <row r="20" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="38"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="24" t="s">
         <v>25</v>
       </c>
@@ -3760,8 +3766,8 @@
       <c r="BB20" s="5"/>
       <c r="BC20" s="5"/>
       <c r="BD20" s="5"/>
-      <c r="BE20" s="11"/>
-      <c r="BF20" s="12"/>
+      <c r="BE20" s="50"/>
+      <c r="BF20" s="51"/>
       <c r="BG20" s="6"/>
       <c r="BH20" s="5"/>
       <c r="BI20" s="5"/>
@@ -3853,7 +3859,7 @@
       <c r="EQ20" s="3"/>
     </row>
     <row r="21" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="38"/>
+      <c r="A21" s="44"/>
       <c r="B21" s="22" t="s">
         <v>26</v>
       </c>
@@ -3913,14 +3919,14 @@
       <c r="BD21" s="5"/>
       <c r="BE21" s="5"/>
       <c r="BF21" s="7"/>
-      <c r="BG21" s="10"/>
-      <c r="BH21" s="11"/>
-      <c r="BI21" s="11"/>
-      <c r="BJ21" s="11"/>
-      <c r="BK21" s="11"/>
-      <c r="BL21" s="11"/>
-      <c r="BM21" s="11"/>
-      <c r="BN21" s="11"/>
+      <c r="BG21" s="49"/>
+      <c r="BH21" s="50"/>
+      <c r="BI21" s="50"/>
+      <c r="BJ21" s="50"/>
+      <c r="BK21" s="50"/>
+      <c r="BL21" s="50"/>
+      <c r="BM21" s="50"/>
+      <c r="BN21" s="50"/>
       <c r="BO21" s="5"/>
       <c r="BP21" s="5"/>
       <c r="BQ21" s="5"/>
@@ -4004,7 +4010,7 @@
       <c r="EQ21" s="3"/>
     </row>
     <row r="22" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="38"/>
+      <c r="A22" s="44"/>
       <c r="B22" s="24" t="s">
         <v>27</v>
       </c>
@@ -4072,10 +4078,10 @@
       <c r="BL22" s="5"/>
       <c r="BM22" s="5"/>
       <c r="BN22" s="5"/>
-      <c r="BO22" s="11"/>
-      <c r="BP22" s="11"/>
-      <c r="BQ22" s="11"/>
-      <c r="BR22" s="11"/>
+      <c r="BO22" s="50"/>
+      <c r="BP22" s="50"/>
+      <c r="BQ22" s="50"/>
+      <c r="BR22" s="50"/>
       <c r="BS22" s="5"/>
       <c r="BT22" s="7"/>
       <c r="BU22" s="6"/>
@@ -4155,7 +4161,7 @@
       <c r="EQ22" s="3"/>
     </row>
     <row r="23" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="23" t="s">
         <v>28</v>
       </c>
@@ -4227,8 +4233,8 @@
       <c r="BP23" s="5"/>
       <c r="BQ23" s="5"/>
       <c r="BR23" s="5"/>
-      <c r="BS23" s="11"/>
-      <c r="BT23" s="12"/>
+      <c r="BS23" s="50"/>
+      <c r="BT23" s="51"/>
       <c r="BU23" s="6"/>
       <c r="BV23" s="5"/>
       <c r="BW23" s="5"/>
@@ -4306,7 +4312,7 @@
       <c r="EQ23" s="3"/>
     </row>
     <row r="24" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="39" t="s">
+      <c r="A24" s="47" t="s">
         <v>44</v>
       </c>
       <c r="B24" s="24" t="s">
@@ -4382,14 +4388,14 @@
       <c r="BR24" s="5"/>
       <c r="BS24" s="5"/>
       <c r="BT24" s="7"/>
-      <c r="BU24" s="10"/>
-      <c r="BV24" s="11"/>
-      <c r="BW24" s="11"/>
-      <c r="BX24" s="11"/>
-      <c r="BY24" s="11"/>
-      <c r="BZ24" s="11"/>
-      <c r="CA24" s="11"/>
-      <c r="CB24" s="11"/>
+      <c r="BU24" s="49"/>
+      <c r="BV24" s="50"/>
+      <c r="BW24" s="50"/>
+      <c r="BX24" s="50"/>
+      <c r="BY24" s="50"/>
+      <c r="BZ24" s="50"/>
+      <c r="CA24" s="50"/>
+      <c r="CB24" s="50"/>
       <c r="CC24" s="5"/>
       <c r="CD24" s="5"/>
       <c r="CE24" s="5"/>
@@ -4440,7 +4446,7 @@
       <c r="DX24" s="7"/>
     </row>
     <row r="25" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="22" t="s">
         <v>30</v>
       </c>
@@ -4522,12 +4528,12 @@
       <c r="BZ25" s="5"/>
       <c r="CA25" s="5"/>
       <c r="CB25" s="5"/>
-      <c r="CC25" s="11"/>
-      <c r="CD25" s="11"/>
-      <c r="CE25" s="11"/>
-      <c r="CF25" s="11"/>
-      <c r="CG25" s="11"/>
-      <c r="CH25" s="12"/>
+      <c r="CC25" s="50"/>
+      <c r="CD25" s="50"/>
+      <c r="CE25" s="50"/>
+      <c r="CF25" s="50"/>
+      <c r="CG25" s="50"/>
+      <c r="CH25" s="51"/>
       <c r="CI25" s="6"/>
       <c r="CJ25" s="5"/>
       <c r="CK25" s="5"/>
@@ -4591,7 +4597,7 @@
       <c r="EQ25" s="3"/>
     </row>
     <row r="26" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="39"/>
+      <c r="A26" s="47"/>
       <c r="B26" s="24" t="s">
         <v>31</v>
       </c>
@@ -4679,10 +4685,10 @@
       <c r="CF26" s="5"/>
       <c r="CG26" s="5"/>
       <c r="CH26" s="7"/>
-      <c r="CI26" s="10"/>
-      <c r="CJ26" s="11"/>
-      <c r="CK26" s="11"/>
-      <c r="CL26" s="11"/>
+      <c r="CI26" s="49"/>
+      <c r="CJ26" s="50"/>
+      <c r="CK26" s="50"/>
+      <c r="CL26" s="50"/>
       <c r="CM26" s="5"/>
       <c r="CN26" s="5"/>
       <c r="CO26" s="5"/>
@@ -4723,7 +4729,7 @@
       <c r="DX26" s="7"/>
     </row>
     <row r="27" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="39"/>
+      <c r="A27" s="47"/>
       <c r="B27" s="22" t="s">
         <v>32</v>
       </c>
@@ -4815,12 +4821,12 @@
       <c r="CJ27" s="5"/>
       <c r="CK27" s="5"/>
       <c r="CL27" s="5"/>
-      <c r="CM27" s="11"/>
-      <c r="CN27" s="11"/>
-      <c r="CO27" s="11"/>
-      <c r="CP27" s="11"/>
-      <c r="CQ27" s="11"/>
-      <c r="CR27" s="11"/>
+      <c r="CM27" s="50"/>
+      <c r="CN27" s="50"/>
+      <c r="CO27" s="50"/>
+      <c r="CP27" s="50"/>
+      <c r="CQ27" s="50"/>
+      <c r="CR27" s="50"/>
       <c r="CS27" s="5"/>
       <c r="CT27" s="5"/>
       <c r="CU27" s="5"/>
@@ -4874,7 +4880,7 @@
       <c r="EQ27" s="3"/>
     </row>
     <row r="28" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="24" t="s">
         <v>33</v>
       </c>
@@ -4972,10 +4978,10 @@
       <c r="CP28" s="5"/>
       <c r="CQ28" s="5"/>
       <c r="CR28" s="5"/>
-      <c r="CS28" s="11"/>
-      <c r="CT28" s="11"/>
-      <c r="CU28" s="11"/>
-      <c r="CV28" s="12"/>
+      <c r="CS28" s="50"/>
+      <c r="CT28" s="50"/>
+      <c r="CU28" s="50"/>
+      <c r="CV28" s="51"/>
       <c r="CW28" s="6"/>
       <c r="CX28" s="5"/>
       <c r="CY28" s="5"/>
@@ -5006,7 +5012,7 @@
       <c r="DX28" s="7"/>
     </row>
     <row r="29" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="22" t="s">
         <v>34</v>
       </c>
@@ -5108,12 +5114,12 @@
       <c r="CT29" s="5"/>
       <c r="CU29" s="5"/>
       <c r="CV29" s="7"/>
-      <c r="CW29" s="10"/>
-      <c r="CX29" s="11"/>
-      <c r="CY29" s="11"/>
-      <c r="CZ29" s="11"/>
-      <c r="DA29" s="11"/>
-      <c r="DB29" s="11"/>
+      <c r="CW29" s="49"/>
+      <c r="CX29" s="50"/>
+      <c r="CY29" s="50"/>
+      <c r="CZ29" s="50"/>
+      <c r="DA29" s="50"/>
+      <c r="DB29" s="50"/>
       <c r="DC29" s="5"/>
       <c r="DD29" s="5"/>
       <c r="DE29" s="5"/>
@@ -5157,7 +5163,7 @@
       <c r="EQ29" s="3"/>
     </row>
     <row r="30" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="39"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="24" t="s">
         <v>35</v>
       </c>
@@ -5265,10 +5271,10 @@
       <c r="CZ30" s="5"/>
       <c r="DA30" s="5"/>
       <c r="DB30" s="5"/>
-      <c r="DC30" s="11"/>
-      <c r="DD30" s="11"/>
-      <c r="DE30" s="11"/>
-      <c r="DF30" s="11"/>
+      <c r="DC30" s="50"/>
+      <c r="DD30" s="50"/>
+      <c r="DE30" s="50"/>
+      <c r="DF30" s="50"/>
       <c r="DG30" s="5"/>
       <c r="DH30" s="5"/>
       <c r="DI30" s="5"/>
@@ -5289,7 +5295,7 @@
       <c r="DX30" s="7"/>
     </row>
     <row r="31" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="39"/>
+      <c r="A31" s="47"/>
       <c r="B31" s="22" t="s">
         <v>36</v>
       </c>
@@ -5401,10 +5407,10 @@
       <c r="DD31" s="5"/>
       <c r="DE31" s="5"/>
       <c r="DF31" s="5"/>
-      <c r="DG31" s="11"/>
-      <c r="DH31" s="11"/>
-      <c r="DI31" s="11"/>
-      <c r="DJ31" s="12"/>
+      <c r="DG31" s="50"/>
+      <c r="DH31" s="50"/>
+      <c r="DI31" s="50"/>
+      <c r="DJ31" s="51"/>
       <c r="DK31" s="6"/>
       <c r="DL31" s="5"/>
       <c r="DM31" s="5"/>
@@ -5440,7 +5446,7 @@
       <c r="EQ31" s="3"/>
     </row>
     <row r="32" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="39"/>
+      <c r="A32" s="47"/>
       <c r="B32" s="24" t="s">
         <v>37</v>
       </c>
@@ -5556,12 +5562,12 @@
       <c r="DH32" s="8"/>
       <c r="DI32" s="8"/>
       <c r="DJ32" s="16"/>
-      <c r="DK32" s="10"/>
-      <c r="DL32" s="11"/>
-      <c r="DM32" s="11"/>
-      <c r="DN32" s="11"/>
-      <c r="DO32" s="11"/>
-      <c r="DP32" s="11"/>
+      <c r="DK32" s="49"/>
+      <c r="DL32" s="50"/>
+      <c r="DM32" s="50"/>
+      <c r="DN32" s="50"/>
+      <c r="DO32" s="50"/>
+      <c r="DP32" s="50"/>
       <c r="DQ32" s="8"/>
       <c r="DR32" s="8"/>
       <c r="DS32" s="8"/>
@@ -5572,7 +5578,7 @@
       <c r="DX32" s="16"/>
     </row>
     <row r="33" spans="1:128" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="39"/>
+      <c r="A33" s="47"/>
       <c r="B33" s="22" t="s">
         <v>38</v>
       </c>
@@ -5694,17 +5700,17 @@
       <c r="DN33" s="5"/>
       <c r="DO33" s="5"/>
       <c r="DP33" s="5"/>
-      <c r="DQ33" s="11"/>
-      <c r="DR33" s="11"/>
-      <c r="DS33" s="11"/>
-      <c r="DT33" s="11"/>
+      <c r="DQ33" s="50"/>
+      <c r="DR33" s="50"/>
+      <c r="DS33" s="50"/>
+      <c r="DT33" s="50"/>
       <c r="DU33" s="5"/>
       <c r="DV33" s="5"/>
       <c r="DW33" s="5"/>
       <c r="DX33" s="7"/>
     </row>
     <row r="34" spans="1:128" s="3" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="40"/>
+      <c r="A34" s="48"/>
       <c r="B34" s="26" t="s">
         <v>39</v>
       </c>
@@ -5830,10 +5836,10 @@
       <c r="DR34" s="31"/>
       <c r="DS34" s="31"/>
       <c r="DT34" s="31"/>
-      <c r="DU34" s="33"/>
-      <c r="DV34" s="33"/>
-      <c r="DW34" s="33"/>
-      <c r="DX34" s="34"/>
+      <c r="DU34" s="52"/>
+      <c r="DV34" s="52"/>
+      <c r="DW34" s="52"/>
+      <c r="DX34" s="53"/>
     </row>
     <row r="35" spans="1:128" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="20"/>
@@ -6876,6 +6882,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A12:A23"/>
+    <mergeCell ref="A24:A34"/>
+    <mergeCell ref="BG2:BT4"/>
+    <mergeCell ref="BU2:CH4"/>
+    <mergeCell ref="CI2:CV4"/>
     <mergeCell ref="CW2:DJ4"/>
     <mergeCell ref="DK2:DX4"/>
     <mergeCell ref="A8:A11"/>
@@ -6885,11 +6896,6 @@
     <mergeCell ref="Q2:AD4"/>
     <mergeCell ref="AE2:AR4"/>
     <mergeCell ref="AS2:BF4"/>
-    <mergeCell ref="A12:A23"/>
-    <mergeCell ref="A24:A34"/>
-    <mergeCell ref="BG2:BT4"/>
-    <mergeCell ref="BU2:CH4"/>
-    <mergeCell ref="CI2:CV4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -6907,10 +6913,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:147" ht="33" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="49"/>
+      <c r="B1" s="45"/>
       <c r="DY1" s="3"/>
       <c r="DZ1" s="3"/>
       <c r="EA1" s="3"/>
@@ -6932,154 +6938,154 @@
       <c r="EQ1" s="3"/>
     </row>
     <row r="2" spans="1:147" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="41" t="s">
+      <c r="B2" s="46"/>
+      <c r="C2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="42"/>
-      <c r="O2" s="42"/>
-      <c r="P2" s="42"/>
-      <c r="Q2" s="41" t="s">
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="42"/>
-      <c r="S2" s="42"/>
-      <c r="T2" s="42"/>
-      <c r="U2" s="42"/>
-      <c r="V2" s="42"/>
-      <c r="W2" s="42"/>
-      <c r="X2" s="42"/>
-      <c r="Y2" s="42"/>
-      <c r="Z2" s="42"/>
-      <c r="AA2" s="42"/>
-      <c r="AB2" s="42"/>
-      <c r="AC2" s="42"/>
-      <c r="AD2" s="42"/>
-      <c r="AE2" s="41" t="s">
+      <c r="R2" s="37"/>
+      <c r="S2" s="37"/>
+      <c r="T2" s="37"/>
+      <c r="U2" s="37"/>
+      <c r="V2" s="37"/>
+      <c r="W2" s="37"/>
+      <c r="X2" s="37"/>
+      <c r="Y2" s="37"/>
+      <c r="Z2" s="37"/>
+      <c r="AA2" s="37"/>
+      <c r="AB2" s="37"/>
+      <c r="AC2" s="37"/>
+      <c r="AD2" s="37"/>
+      <c r="AE2" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="AF2" s="42"/>
-      <c r="AG2" s="42"/>
-      <c r="AH2" s="42"/>
-      <c r="AI2" s="42"/>
-      <c r="AJ2" s="42"/>
-      <c r="AK2" s="42"/>
-      <c r="AL2" s="42"/>
-      <c r="AM2" s="42"/>
-      <c r="AN2" s="42"/>
-      <c r="AO2" s="42"/>
-      <c r="AP2" s="42"/>
-      <c r="AQ2" s="42"/>
-      <c r="AR2" s="42"/>
-      <c r="AS2" s="41" t="s">
+      <c r="AF2" s="37"/>
+      <c r="AG2" s="37"/>
+      <c r="AH2" s="37"/>
+      <c r="AI2" s="37"/>
+      <c r="AJ2" s="37"/>
+      <c r="AK2" s="37"/>
+      <c r="AL2" s="37"/>
+      <c r="AM2" s="37"/>
+      <c r="AN2" s="37"/>
+      <c r="AO2" s="37"/>
+      <c r="AP2" s="37"/>
+      <c r="AQ2" s="37"/>
+      <c r="AR2" s="37"/>
+      <c r="AS2" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="AT2" s="42"/>
-      <c r="AU2" s="42"/>
-      <c r="AV2" s="42"/>
-      <c r="AW2" s="42"/>
-      <c r="AX2" s="42"/>
-      <c r="AY2" s="42"/>
-      <c r="AZ2" s="42"/>
-      <c r="BA2" s="42"/>
-      <c r="BB2" s="42"/>
-      <c r="BC2" s="42"/>
-      <c r="BD2" s="42"/>
-      <c r="BE2" s="42"/>
-      <c r="BF2" s="42"/>
-      <c r="BG2" s="41" t="s">
+      <c r="AT2" s="37"/>
+      <c r="AU2" s="37"/>
+      <c r="AV2" s="37"/>
+      <c r="AW2" s="37"/>
+      <c r="AX2" s="37"/>
+      <c r="AY2" s="37"/>
+      <c r="AZ2" s="37"/>
+      <c r="BA2" s="37"/>
+      <c r="BB2" s="37"/>
+      <c r="BC2" s="37"/>
+      <c r="BD2" s="37"/>
+      <c r="BE2" s="37"/>
+      <c r="BF2" s="37"/>
+      <c r="BG2" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="BH2" s="42"/>
-      <c r="BI2" s="42"/>
-      <c r="BJ2" s="42"/>
-      <c r="BK2" s="42"/>
-      <c r="BL2" s="42"/>
-      <c r="BM2" s="42"/>
-      <c r="BN2" s="42"/>
-      <c r="BO2" s="42"/>
-      <c r="BP2" s="42"/>
-      <c r="BQ2" s="42"/>
-      <c r="BR2" s="42"/>
-      <c r="BS2" s="42"/>
-      <c r="BT2" s="42"/>
-      <c r="BU2" s="41" t="s">
+      <c r="BH2" s="37"/>
+      <c r="BI2" s="37"/>
+      <c r="BJ2" s="37"/>
+      <c r="BK2" s="37"/>
+      <c r="BL2" s="37"/>
+      <c r="BM2" s="37"/>
+      <c r="BN2" s="37"/>
+      <c r="BO2" s="37"/>
+      <c r="BP2" s="37"/>
+      <c r="BQ2" s="37"/>
+      <c r="BR2" s="37"/>
+      <c r="BS2" s="37"/>
+      <c r="BT2" s="37"/>
+      <c r="BU2" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="BV2" s="42"/>
-      <c r="BW2" s="42"/>
-      <c r="BX2" s="42"/>
-      <c r="BY2" s="42"/>
-      <c r="BZ2" s="42"/>
-      <c r="CA2" s="42"/>
-      <c r="CB2" s="42"/>
-      <c r="CC2" s="42"/>
-      <c r="CD2" s="42"/>
-      <c r="CE2" s="42"/>
-      <c r="CF2" s="42"/>
-      <c r="CG2" s="42"/>
-      <c r="CH2" s="42"/>
-      <c r="CI2" s="41" t="s">
+      <c r="BV2" s="37"/>
+      <c r="BW2" s="37"/>
+      <c r="BX2" s="37"/>
+      <c r="BY2" s="37"/>
+      <c r="BZ2" s="37"/>
+      <c r="CA2" s="37"/>
+      <c r="CB2" s="37"/>
+      <c r="CC2" s="37"/>
+      <c r="CD2" s="37"/>
+      <c r="CE2" s="37"/>
+      <c r="CF2" s="37"/>
+      <c r="CG2" s="37"/>
+      <c r="CH2" s="37"/>
+      <c r="CI2" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="CJ2" s="42"/>
-      <c r="CK2" s="42"/>
-      <c r="CL2" s="42"/>
-      <c r="CM2" s="42"/>
-      <c r="CN2" s="42"/>
-      <c r="CO2" s="42"/>
-      <c r="CP2" s="42"/>
-      <c r="CQ2" s="42"/>
-      <c r="CR2" s="42"/>
-      <c r="CS2" s="42"/>
-      <c r="CT2" s="42"/>
-      <c r="CU2" s="42"/>
-      <c r="CV2" s="42"/>
-      <c r="CW2" s="41" t="s">
+      <c r="CJ2" s="37"/>
+      <c r="CK2" s="37"/>
+      <c r="CL2" s="37"/>
+      <c r="CM2" s="37"/>
+      <c r="CN2" s="37"/>
+      <c r="CO2" s="37"/>
+      <c r="CP2" s="37"/>
+      <c r="CQ2" s="37"/>
+      <c r="CR2" s="37"/>
+      <c r="CS2" s="37"/>
+      <c r="CT2" s="37"/>
+      <c r="CU2" s="37"/>
+      <c r="CV2" s="37"/>
+      <c r="CW2" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="CX2" s="42"/>
-      <c r="CY2" s="42"/>
-      <c r="CZ2" s="42"/>
-      <c r="DA2" s="42"/>
-      <c r="DB2" s="42"/>
-      <c r="DC2" s="42"/>
-      <c r="DD2" s="42"/>
-      <c r="DE2" s="42"/>
-      <c r="DF2" s="42"/>
-      <c r="DG2" s="42"/>
-      <c r="DH2" s="42"/>
-      <c r="DI2" s="42"/>
-      <c r="DJ2" s="42"/>
-      <c r="DK2" s="47" t="s">
+      <c r="CX2" s="37"/>
+      <c r="CY2" s="37"/>
+      <c r="CZ2" s="37"/>
+      <c r="DA2" s="37"/>
+      <c r="DB2" s="37"/>
+      <c r="DC2" s="37"/>
+      <c r="DD2" s="37"/>
+      <c r="DE2" s="37"/>
+      <c r="DF2" s="37"/>
+      <c r="DG2" s="37"/>
+      <c r="DH2" s="37"/>
+      <c r="DI2" s="37"/>
+      <c r="DJ2" s="37"/>
+      <c r="DK2" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="DL2" s="47"/>
-      <c r="DM2" s="47"/>
-      <c r="DN2" s="47"/>
-      <c r="DO2" s="47"/>
-      <c r="DP2" s="47"/>
-      <c r="DQ2" s="47"/>
-      <c r="DR2" s="47"/>
-      <c r="DS2" s="47"/>
-      <c r="DT2" s="47"/>
-      <c r="DU2" s="47"/>
-      <c r="DV2" s="47"/>
-      <c r="DW2" s="47"/>
-      <c r="DX2" s="47"/>
+      <c r="DL2" s="42"/>
+      <c r="DM2" s="42"/>
+      <c r="DN2" s="42"/>
+      <c r="DO2" s="42"/>
+      <c r="DP2" s="42"/>
+      <c r="DQ2" s="42"/>
+      <c r="DR2" s="42"/>
+      <c r="DS2" s="42"/>
+      <c r="DT2" s="42"/>
+      <c r="DU2" s="42"/>
+      <c r="DV2" s="42"/>
+      <c r="DW2" s="42"/>
+      <c r="DX2" s="42"/>
       <c r="DY2" s="3"/>
       <c r="DZ2" s="3"/>
       <c r="EA2" s="3"/>
@@ -7101,134 +7107,134 @@
       <c r="EQ2" s="3"/>
     </row>
     <row r="3" spans="1:147" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50"/>
-      <c r="B3" s="50"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="44"/>
-      <c r="Q3" s="43"/>
-      <c r="R3" s="44"/>
-      <c r="S3" s="44"/>
-      <c r="T3" s="44"/>
-      <c r="U3" s="44"/>
-      <c r="V3" s="44"/>
-      <c r="W3" s="44"/>
-      <c r="X3" s="44"/>
-      <c r="Y3" s="44"/>
-      <c r="Z3" s="44"/>
-      <c r="AA3" s="44"/>
-      <c r="AB3" s="44"/>
-      <c r="AC3" s="44"/>
-      <c r="AD3" s="44"/>
-      <c r="AE3" s="43"/>
-      <c r="AF3" s="44"/>
-      <c r="AG3" s="44"/>
-      <c r="AH3" s="44"/>
-      <c r="AI3" s="44"/>
-      <c r="AJ3" s="44"/>
-      <c r="AK3" s="44"/>
-      <c r="AL3" s="44"/>
-      <c r="AM3" s="44"/>
-      <c r="AN3" s="44"/>
-      <c r="AO3" s="44"/>
-      <c r="AP3" s="44"/>
-      <c r="AQ3" s="44"/>
-      <c r="AR3" s="44"/>
-      <c r="AS3" s="43"/>
-      <c r="AT3" s="44"/>
-      <c r="AU3" s="44"/>
-      <c r="AV3" s="44"/>
-      <c r="AW3" s="44"/>
-      <c r="AX3" s="44"/>
-      <c r="AY3" s="44"/>
-      <c r="AZ3" s="44"/>
-      <c r="BA3" s="44"/>
-      <c r="BB3" s="44"/>
-      <c r="BC3" s="44"/>
-      <c r="BD3" s="44"/>
-      <c r="BE3" s="44"/>
-      <c r="BF3" s="44"/>
-      <c r="BG3" s="43"/>
-      <c r="BH3" s="44"/>
-      <c r="BI3" s="44"/>
-      <c r="BJ3" s="44"/>
-      <c r="BK3" s="44"/>
-      <c r="BL3" s="44"/>
-      <c r="BM3" s="44"/>
-      <c r="BN3" s="44"/>
-      <c r="BO3" s="44"/>
-      <c r="BP3" s="44"/>
-      <c r="BQ3" s="44"/>
-      <c r="BR3" s="44"/>
-      <c r="BS3" s="44"/>
-      <c r="BT3" s="44"/>
-      <c r="BU3" s="43"/>
-      <c r="BV3" s="44"/>
-      <c r="BW3" s="44"/>
-      <c r="BX3" s="44"/>
-      <c r="BY3" s="44"/>
-      <c r="BZ3" s="44"/>
-      <c r="CA3" s="44"/>
-      <c r="CB3" s="44"/>
-      <c r="CC3" s="44"/>
-      <c r="CD3" s="44"/>
-      <c r="CE3" s="44"/>
-      <c r="CF3" s="44"/>
-      <c r="CG3" s="44"/>
-      <c r="CH3" s="44"/>
-      <c r="CI3" s="43"/>
-      <c r="CJ3" s="44"/>
-      <c r="CK3" s="44"/>
-      <c r="CL3" s="44"/>
-      <c r="CM3" s="44"/>
-      <c r="CN3" s="44"/>
-      <c r="CO3" s="44"/>
-      <c r="CP3" s="44"/>
-      <c r="CQ3" s="44"/>
-      <c r="CR3" s="44"/>
-      <c r="CS3" s="44"/>
-      <c r="CT3" s="44"/>
-      <c r="CU3" s="44"/>
-      <c r="CV3" s="44"/>
-      <c r="CW3" s="43"/>
-      <c r="CX3" s="44"/>
-      <c r="CY3" s="44"/>
-      <c r="CZ3" s="44"/>
-      <c r="DA3" s="44"/>
-      <c r="DB3" s="44"/>
-      <c r="DC3" s="44"/>
-      <c r="DD3" s="44"/>
-      <c r="DE3" s="44"/>
-      <c r="DF3" s="44"/>
-      <c r="DG3" s="44"/>
-      <c r="DH3" s="44"/>
-      <c r="DI3" s="44"/>
-      <c r="DJ3" s="44"/>
-      <c r="DK3" s="47"/>
-      <c r="DL3" s="47"/>
-      <c r="DM3" s="47"/>
-      <c r="DN3" s="47"/>
-      <c r="DO3" s="47"/>
-      <c r="DP3" s="47"/>
-      <c r="DQ3" s="47"/>
-      <c r="DR3" s="47"/>
-      <c r="DS3" s="47"/>
-      <c r="DT3" s="47"/>
-      <c r="DU3" s="47"/>
-      <c r="DV3" s="47"/>
-      <c r="DW3" s="47"/>
-      <c r="DX3" s="47"/>
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="38"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="39"/>
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="38"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="39"/>
+      <c r="AH3" s="39"/>
+      <c r="AI3" s="39"/>
+      <c r="AJ3" s="39"/>
+      <c r="AK3" s="39"/>
+      <c r="AL3" s="39"/>
+      <c r="AM3" s="39"/>
+      <c r="AN3" s="39"/>
+      <c r="AO3" s="39"/>
+      <c r="AP3" s="39"/>
+      <c r="AQ3" s="39"/>
+      <c r="AR3" s="39"/>
+      <c r="AS3" s="38"/>
+      <c r="AT3" s="39"/>
+      <c r="AU3" s="39"/>
+      <c r="AV3" s="39"/>
+      <c r="AW3" s="39"/>
+      <c r="AX3" s="39"/>
+      <c r="AY3" s="39"/>
+      <c r="AZ3" s="39"/>
+      <c r="BA3" s="39"/>
+      <c r="BB3" s="39"/>
+      <c r="BC3" s="39"/>
+      <c r="BD3" s="39"/>
+      <c r="BE3" s="39"/>
+      <c r="BF3" s="39"/>
+      <c r="BG3" s="38"/>
+      <c r="BH3" s="39"/>
+      <c r="BI3" s="39"/>
+      <c r="BJ3" s="39"/>
+      <c r="BK3" s="39"/>
+      <c r="BL3" s="39"/>
+      <c r="BM3" s="39"/>
+      <c r="BN3" s="39"/>
+      <c r="BO3" s="39"/>
+      <c r="BP3" s="39"/>
+      <c r="BQ3" s="39"/>
+      <c r="BR3" s="39"/>
+      <c r="BS3" s="39"/>
+      <c r="BT3" s="39"/>
+      <c r="BU3" s="38"/>
+      <c r="BV3" s="39"/>
+      <c r="BW3" s="39"/>
+      <c r="BX3" s="39"/>
+      <c r="BY3" s="39"/>
+      <c r="BZ3" s="39"/>
+      <c r="CA3" s="39"/>
+      <c r="CB3" s="39"/>
+      <c r="CC3" s="39"/>
+      <c r="CD3" s="39"/>
+      <c r="CE3" s="39"/>
+      <c r="CF3" s="39"/>
+      <c r="CG3" s="39"/>
+      <c r="CH3" s="39"/>
+      <c r="CI3" s="38"/>
+      <c r="CJ3" s="39"/>
+      <c r="CK3" s="39"/>
+      <c r="CL3" s="39"/>
+      <c r="CM3" s="39"/>
+      <c r="CN3" s="39"/>
+      <c r="CO3" s="39"/>
+      <c r="CP3" s="39"/>
+      <c r="CQ3" s="39"/>
+      <c r="CR3" s="39"/>
+      <c r="CS3" s="39"/>
+      <c r="CT3" s="39"/>
+      <c r="CU3" s="39"/>
+      <c r="CV3" s="39"/>
+      <c r="CW3" s="38"/>
+      <c r="CX3" s="39"/>
+      <c r="CY3" s="39"/>
+      <c r="CZ3" s="39"/>
+      <c r="DA3" s="39"/>
+      <c r="DB3" s="39"/>
+      <c r="DC3" s="39"/>
+      <c r="DD3" s="39"/>
+      <c r="DE3" s="39"/>
+      <c r="DF3" s="39"/>
+      <c r="DG3" s="39"/>
+      <c r="DH3" s="39"/>
+      <c r="DI3" s="39"/>
+      <c r="DJ3" s="39"/>
+      <c r="DK3" s="42"/>
+      <c r="DL3" s="42"/>
+      <c r="DM3" s="42"/>
+      <c r="DN3" s="42"/>
+      <c r="DO3" s="42"/>
+      <c r="DP3" s="42"/>
+      <c r="DQ3" s="42"/>
+      <c r="DR3" s="42"/>
+      <c r="DS3" s="42"/>
+      <c r="DT3" s="42"/>
+      <c r="DU3" s="42"/>
+      <c r="DV3" s="42"/>
+      <c r="DW3" s="42"/>
+      <c r="DX3" s="42"/>
       <c r="DY3" s="3"/>
       <c r="DZ3" s="3"/>
       <c r="EA3" s="3"/>
@@ -7250,134 +7256,134 @@
       <c r="EQ3" s="3"/>
     </row>
     <row r="4" spans="1:147" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="50"/>
-      <c r="B4" s="50"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
-      <c r="M4" s="46"/>
-      <c r="N4" s="46"/>
-      <c r="O4" s="46"/>
-      <c r="P4" s="46"/>
-      <c r="Q4" s="45"/>
-      <c r="R4" s="46"/>
-      <c r="S4" s="46"/>
-      <c r="T4" s="46"/>
-      <c r="U4" s="46"/>
-      <c r="V4" s="46"/>
-      <c r="W4" s="46"/>
-      <c r="X4" s="46"/>
-      <c r="Y4" s="46"/>
-      <c r="Z4" s="46"/>
-      <c r="AA4" s="46"/>
-      <c r="AB4" s="46"/>
-      <c r="AC4" s="46"/>
-      <c r="AD4" s="46"/>
-      <c r="AE4" s="45"/>
-      <c r="AF4" s="46"/>
-      <c r="AG4" s="46"/>
-      <c r="AH4" s="46"/>
-      <c r="AI4" s="46"/>
-      <c r="AJ4" s="46"/>
-      <c r="AK4" s="46"/>
-      <c r="AL4" s="46"/>
-      <c r="AM4" s="46"/>
-      <c r="AN4" s="46"/>
-      <c r="AO4" s="46"/>
-      <c r="AP4" s="46"/>
-      <c r="AQ4" s="46"/>
-      <c r="AR4" s="46"/>
-      <c r="AS4" s="45"/>
-      <c r="AT4" s="46"/>
-      <c r="AU4" s="46"/>
-      <c r="AV4" s="46"/>
-      <c r="AW4" s="46"/>
-      <c r="AX4" s="46"/>
-      <c r="AY4" s="46"/>
-      <c r="AZ4" s="46"/>
-      <c r="BA4" s="46"/>
-      <c r="BB4" s="46"/>
-      <c r="BC4" s="46"/>
-      <c r="BD4" s="46"/>
-      <c r="BE4" s="46"/>
-      <c r="BF4" s="46"/>
-      <c r="BG4" s="45"/>
-      <c r="BH4" s="46"/>
-      <c r="BI4" s="46"/>
-      <c r="BJ4" s="46"/>
-      <c r="BK4" s="46"/>
-      <c r="BL4" s="46"/>
-      <c r="BM4" s="46"/>
-      <c r="BN4" s="46"/>
-      <c r="BO4" s="46"/>
-      <c r="BP4" s="46"/>
-      <c r="BQ4" s="46"/>
-      <c r="BR4" s="46"/>
-      <c r="BS4" s="46"/>
-      <c r="BT4" s="46"/>
-      <c r="BU4" s="45"/>
-      <c r="BV4" s="46"/>
-      <c r="BW4" s="46"/>
-      <c r="BX4" s="46"/>
-      <c r="BY4" s="46"/>
-      <c r="BZ4" s="46"/>
-      <c r="CA4" s="46"/>
-      <c r="CB4" s="46"/>
-      <c r="CC4" s="46"/>
-      <c r="CD4" s="46"/>
-      <c r="CE4" s="46"/>
-      <c r="CF4" s="46"/>
-      <c r="CG4" s="46"/>
-      <c r="CH4" s="46"/>
-      <c r="CI4" s="45"/>
-      <c r="CJ4" s="46"/>
-      <c r="CK4" s="46"/>
-      <c r="CL4" s="46"/>
-      <c r="CM4" s="46"/>
-      <c r="CN4" s="46"/>
-      <c r="CO4" s="46"/>
-      <c r="CP4" s="46"/>
-      <c r="CQ4" s="46"/>
-      <c r="CR4" s="46"/>
-      <c r="CS4" s="46"/>
-      <c r="CT4" s="46"/>
-      <c r="CU4" s="46"/>
-      <c r="CV4" s="46"/>
-      <c r="CW4" s="45"/>
-      <c r="CX4" s="46"/>
-      <c r="CY4" s="46"/>
-      <c r="CZ4" s="46"/>
-      <c r="DA4" s="46"/>
-      <c r="DB4" s="46"/>
-      <c r="DC4" s="46"/>
-      <c r="DD4" s="46"/>
-      <c r="DE4" s="46"/>
-      <c r="DF4" s="46"/>
-      <c r="DG4" s="46"/>
-      <c r="DH4" s="46"/>
-      <c r="DI4" s="46"/>
-      <c r="DJ4" s="46"/>
-      <c r="DK4" s="47"/>
-      <c r="DL4" s="47"/>
-      <c r="DM4" s="47"/>
-      <c r="DN4" s="47"/>
-      <c r="DO4" s="47"/>
-      <c r="DP4" s="47"/>
-      <c r="DQ4" s="47"/>
-      <c r="DR4" s="47"/>
-      <c r="DS4" s="47"/>
-      <c r="DT4" s="47"/>
-      <c r="DU4" s="47"/>
-      <c r="DV4" s="47"/>
-      <c r="DW4" s="47"/>
-      <c r="DX4" s="47"/>
+      <c r="A4" s="46"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="40"/>
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="41"/>
+      <c r="V4" s="41"/>
+      <c r="W4" s="41"/>
+      <c r="X4" s="41"/>
+      <c r="Y4" s="41"/>
+      <c r="Z4" s="41"/>
+      <c r="AA4" s="41"/>
+      <c r="AB4" s="41"/>
+      <c r="AC4" s="41"/>
+      <c r="AD4" s="41"/>
+      <c r="AE4" s="40"/>
+      <c r="AF4" s="41"/>
+      <c r="AG4" s="41"/>
+      <c r="AH4" s="41"/>
+      <c r="AI4" s="41"/>
+      <c r="AJ4" s="41"/>
+      <c r="AK4" s="41"/>
+      <c r="AL4" s="41"/>
+      <c r="AM4" s="41"/>
+      <c r="AN4" s="41"/>
+      <c r="AO4" s="41"/>
+      <c r="AP4" s="41"/>
+      <c r="AQ4" s="41"/>
+      <c r="AR4" s="41"/>
+      <c r="AS4" s="40"/>
+      <c r="AT4" s="41"/>
+      <c r="AU4" s="41"/>
+      <c r="AV4" s="41"/>
+      <c r="AW4" s="41"/>
+      <c r="AX4" s="41"/>
+      <c r="AY4" s="41"/>
+      <c r="AZ4" s="41"/>
+      <c r="BA4" s="41"/>
+      <c r="BB4" s="41"/>
+      <c r="BC4" s="41"/>
+      <c r="BD4" s="41"/>
+      <c r="BE4" s="41"/>
+      <c r="BF4" s="41"/>
+      <c r="BG4" s="40"/>
+      <c r="BH4" s="41"/>
+      <c r="BI4" s="41"/>
+      <c r="BJ4" s="41"/>
+      <c r="BK4" s="41"/>
+      <c r="BL4" s="41"/>
+      <c r="BM4" s="41"/>
+      <c r="BN4" s="41"/>
+      <c r="BO4" s="41"/>
+      <c r="BP4" s="41"/>
+      <c r="BQ4" s="41"/>
+      <c r="BR4" s="41"/>
+      <c r="BS4" s="41"/>
+      <c r="BT4" s="41"/>
+      <c r="BU4" s="40"/>
+      <c r="BV4" s="41"/>
+      <c r="BW4" s="41"/>
+      <c r="BX4" s="41"/>
+      <c r="BY4" s="41"/>
+      <c r="BZ4" s="41"/>
+      <c r="CA4" s="41"/>
+      <c r="CB4" s="41"/>
+      <c r="CC4" s="41"/>
+      <c r="CD4" s="41"/>
+      <c r="CE4" s="41"/>
+      <c r="CF4" s="41"/>
+      <c r="CG4" s="41"/>
+      <c r="CH4" s="41"/>
+      <c r="CI4" s="40"/>
+      <c r="CJ4" s="41"/>
+      <c r="CK4" s="41"/>
+      <c r="CL4" s="41"/>
+      <c r="CM4" s="41"/>
+      <c r="CN4" s="41"/>
+      <c r="CO4" s="41"/>
+      <c r="CP4" s="41"/>
+      <c r="CQ4" s="41"/>
+      <c r="CR4" s="41"/>
+      <c r="CS4" s="41"/>
+      <c r="CT4" s="41"/>
+      <c r="CU4" s="41"/>
+      <c r="CV4" s="41"/>
+      <c r="CW4" s="40"/>
+      <c r="CX4" s="41"/>
+      <c r="CY4" s="41"/>
+      <c r="CZ4" s="41"/>
+      <c r="DA4" s="41"/>
+      <c r="DB4" s="41"/>
+      <c r="DC4" s="41"/>
+      <c r="DD4" s="41"/>
+      <c r="DE4" s="41"/>
+      <c r="DF4" s="41"/>
+      <c r="DG4" s="41"/>
+      <c r="DH4" s="41"/>
+      <c r="DI4" s="41"/>
+      <c r="DJ4" s="41"/>
+      <c r="DK4" s="42"/>
+      <c r="DL4" s="42"/>
+      <c r="DM4" s="42"/>
+      <c r="DN4" s="42"/>
+      <c r="DO4" s="42"/>
+      <c r="DP4" s="42"/>
+      <c r="DQ4" s="42"/>
+      <c r="DR4" s="42"/>
+      <c r="DS4" s="42"/>
+      <c r="DT4" s="42"/>
+      <c r="DU4" s="42"/>
+      <c r="DV4" s="42"/>
+      <c r="DW4" s="42"/>
+      <c r="DX4" s="42"/>
       <c r="DY4" s="3"/>
       <c r="DZ4" s="3"/>
       <c r="EA4" s="3"/>
@@ -7854,7 +7860,7 @@
       <c r="EQ7" s="3"/>
     </row>
     <row r="8" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="43" t="s">
         <v>42</v>
       </c>
       <c r="B8" s="24" t="s">
@@ -8007,7 +8013,7 @@
       <c r="EQ8" s="3"/>
     </row>
     <row r="9" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="38"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="22" t="s">
         <v>20</v>
       </c>
@@ -8016,10 +8022,10 @@
       <c r="E9" s="8"/>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="8"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
@@ -8158,7 +8164,7 @@
       <c r="EQ9" s="3"/>
     </row>
     <row r="10" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="38"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="24" t="s">
         <v>21</v>
       </c>
@@ -8309,15 +8315,15 @@
       <c r="EQ10" s="3"/>
     </row>
     <row r="11" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="38"/>
+      <c r="A11" s="44"/>
       <c r="B11" s="22" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="8"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
@@ -8460,7 +8466,7 @@
       <c r="EQ11" s="3"/>
     </row>
     <row r="12" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="44" t="s">
         <v>43</v>
       </c>
       <c r="B12" s="25" t="s">
@@ -8475,12 +8481,12 @@
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="35"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="33"/>
       <c r="R12" s="13"/>
       <c r="S12" s="13"/>
       <c r="T12" s="13"/>
@@ -8613,7 +8619,7 @@
       <c r="EQ12" s="3"/>
     </row>
     <row r="13" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="38"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="23" t="s">
         <v>15</v>
       </c>
@@ -8631,11 +8637,11 @@
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
       <c r="P13" s="7"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="5"/>
-      <c r="S13" s="5"/>
-      <c r="T13" s="5"/>
-      <c r="U13" s="5"/>
+      <c r="Q13" s="10"/>
+      <c r="R13" s="11"/>
+      <c r="S13" s="11"/>
+      <c r="T13" s="11"/>
+      <c r="U13" s="11"/>
       <c r="V13" s="5"/>
       <c r="W13" s="13"/>
       <c r="X13" s="13"/>
@@ -8764,7 +8770,7 @@
       <c r="EQ13" s="3"/>
     </row>
     <row r="14" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="24" t="s">
         <v>16</v>
       </c>
@@ -8787,15 +8793,15 @@
       <c r="S14" s="5"/>
       <c r="T14" s="5"/>
       <c r="U14" s="5"/>
-      <c r="V14" s="5"/>
-      <c r="W14" s="5"/>
-      <c r="X14" s="5"/>
-      <c r="Y14" s="5"/>
-      <c r="Z14" s="5"/>
-      <c r="AA14" s="5"/>
-      <c r="AB14" s="13"/>
-      <c r="AC14" s="13"/>
-      <c r="AD14" s="14"/>
+      <c r="V14" s="11"/>
+      <c r="W14" s="11"/>
+      <c r="X14" s="11"/>
+      <c r="Y14" s="11"/>
+      <c r="Z14" s="11"/>
+      <c r="AA14" s="11"/>
+      <c r="AB14" s="11"/>
+      <c r="AC14" s="11"/>
+      <c r="AD14" s="12"/>
       <c r="AE14" s="6"/>
       <c r="AF14" s="5"/>
       <c r="AG14" s="5"/>
@@ -8915,7 +8921,7 @@
       <c r="EQ14" s="3"/>
     </row>
     <row r="15" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="22" t="s">
         <v>17</v>
       </c>
@@ -8947,7 +8953,7 @@
       <c r="AB15" s="5"/>
       <c r="AC15" s="5"/>
       <c r="AD15" s="7"/>
-      <c r="AE15" s="35"/>
+      <c r="AE15" s="33"/>
       <c r="AF15" s="13"/>
       <c r="AG15" s="13"/>
       <c r="AH15" s="13"/>
@@ -9066,7 +9072,7 @@
       <c r="EQ15" s="3"/>
     </row>
     <row r="16" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="38"/>
+      <c r="A16" s="44"/>
       <c r="B16" s="25" t="s">
         <v>18</v>
       </c>
@@ -9098,11 +9104,11 @@
       <c r="AB16" s="5"/>
       <c r="AC16" s="5"/>
       <c r="AD16" s="7"/>
-      <c r="AE16" s="6"/>
-      <c r="AF16" s="5"/>
-      <c r="AG16" s="5"/>
-      <c r="AH16" s="5"/>
-      <c r="AI16" s="5"/>
+      <c r="AE16" s="10"/>
+      <c r="AF16" s="11"/>
+      <c r="AG16" s="11"/>
+      <c r="AH16" s="11"/>
+      <c r="AI16" s="11"/>
       <c r="AJ16" s="5"/>
       <c r="AK16" s="5"/>
       <c r="AL16" s="13"/>
@@ -9217,7 +9223,7 @@
       <c r="EQ16" s="3"/>
     </row>
     <row r="17" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="38"/>
+      <c r="A17" s="44"/>
       <c r="B17" s="23" t="s">
         <v>22</v>
       </c>
@@ -9254,10 +9260,10 @@
       <c r="AG17" s="5"/>
       <c r="AH17" s="5"/>
       <c r="AI17" s="5"/>
-      <c r="AJ17" s="5"/>
-      <c r="AK17" s="5"/>
-      <c r="AL17" s="5"/>
-      <c r="AM17" s="5"/>
+      <c r="AJ17" s="11"/>
+      <c r="AK17" s="11"/>
+      <c r="AL17" s="11"/>
+      <c r="AM17" s="11"/>
       <c r="AN17" s="5"/>
       <c r="AO17" s="5"/>
       <c r="AP17" s="5"/>
@@ -9368,9 +9374,9 @@
       <c r="EQ17" s="3"/>
     </row>
     <row r="18" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="38"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="25" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5"/>
@@ -9414,7 +9420,7 @@
       <c r="AP18" s="5"/>
       <c r="AQ18" s="5"/>
       <c r="AR18" s="7"/>
-      <c r="AS18" s="35"/>
+      <c r="AS18" s="33"/>
       <c r="AT18" s="13"/>
       <c r="AU18" s="13"/>
       <c r="AV18" s="13"/>
@@ -9519,7 +9525,7 @@
       <c r="EQ18" s="3"/>
     </row>
     <row r="19" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="22" t="s">
         <v>24</v>
       </c>
@@ -9670,7 +9676,7 @@
       <c r="EQ19" s="3"/>
     </row>
     <row r="20" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="38"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="24" t="s">
         <v>25</v>
       </c>
@@ -9821,7 +9827,7 @@
       <c r="EQ20" s="3"/>
     </row>
     <row r="21" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="38"/>
+      <c r="A21" s="44"/>
       <c r="B21" s="22" t="s">
         <v>26</v>
       </c>
@@ -9881,7 +9887,7 @@
       <c r="BD21" s="5"/>
       <c r="BE21" s="5"/>
       <c r="BF21" s="7"/>
-      <c r="BG21" s="35"/>
+      <c r="BG21" s="33"/>
       <c r="BH21" s="13"/>
       <c r="BI21" s="13"/>
       <c r="BJ21" s="13"/>
@@ -9972,7 +9978,7 @@
       <c r="EQ21" s="3"/>
     </row>
     <row r="22" spans="1:147" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="38"/>
+      <c r="A22" s="44"/>
       <c r="B22" s="24" t="s">
         <v>27</v>
       </c>
@@ -10123,9 +10129,9 @@
       <c r="EQ22" s="3"/>
     </row>
     <row r="23" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="23" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="5"/>
@@ -10274,7 +10280,7 @@
       <c r="EQ23" s="3"/>
     </row>
     <row r="24" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="39" t="s">
+      <c r="A24" s="47" t="s">
         <v>44</v>
       </c>
       <c r="B24" s="24" t="s">
@@ -10350,7 +10356,7 @@
       <c r="BR24" s="5"/>
       <c r="BS24" s="5"/>
       <c r="BT24" s="7"/>
-      <c r="BU24" s="35"/>
+      <c r="BU24" s="33"/>
       <c r="BV24" s="13"/>
       <c r="BW24" s="13"/>
       <c r="BX24" s="13"/>
@@ -10408,7 +10414,7 @@
       <c r="DX24" s="7"/>
     </row>
     <row r="25" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
+      <c r="A25" s="47"/>
       <c r="B25" s="22" t="s">
         <v>30</v>
       </c>
@@ -10559,7 +10565,7 @@
       <c r="EQ25" s="3"/>
     </row>
     <row r="26" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="39"/>
+      <c r="A26" s="47"/>
       <c r="B26" s="24" t="s">
         <v>31</v>
       </c>
@@ -10647,7 +10653,7 @@
       <c r="CF26" s="5"/>
       <c r="CG26" s="5"/>
       <c r="CH26" s="7"/>
-      <c r="CI26" s="35"/>
+      <c r="CI26" s="33"/>
       <c r="CJ26" s="13"/>
       <c r="CK26" s="13"/>
       <c r="CL26" s="13"/>
@@ -10691,7 +10697,7 @@
       <c r="DX26" s="7"/>
     </row>
     <row r="27" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="39"/>
+      <c r="A27" s="47"/>
       <c r="B27" s="22" t="s">
         <v>32</v>
       </c>
@@ -10842,7 +10848,7 @@
       <c r="EQ27" s="3"/>
     </row>
     <row r="28" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
+      <c r="A28" s="47"/>
       <c r="B28" s="24" t="s">
         <v>33</v>
       </c>
@@ -10974,7 +10980,7 @@
       <c r="DX28" s="7"/>
     </row>
     <row r="29" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
+      <c r="A29" s="47"/>
       <c r="B29" s="22" t="s">
         <v>34</v>
       </c>
@@ -11076,7 +11082,7 @@
       <c r="CT29" s="5"/>
       <c r="CU29" s="5"/>
       <c r="CV29" s="7"/>
-      <c r="CW29" s="35"/>
+      <c r="CW29" s="33"/>
       <c r="CX29" s="13"/>
       <c r="CY29" s="13"/>
       <c r="CZ29" s="13"/>
@@ -11125,7 +11131,7 @@
       <c r="EQ29" s="3"/>
     </row>
     <row r="30" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="39"/>
+      <c r="A30" s="47"/>
       <c r="B30" s="24" t="s">
         <v>35</v>
       </c>
@@ -11257,7 +11263,7 @@
       <c r="DX30" s="7"/>
     </row>
     <row r="31" spans="1:147" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="39"/>
+      <c r="A31" s="47"/>
       <c r="B31" s="22" t="s">
         <v>36</v>
       </c>
@@ -11408,7 +11414,7 @@
       <c r="EQ31" s="3"/>
     </row>
     <row r="32" spans="1:147" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="39"/>
+      <c r="A32" s="47"/>
       <c r="B32" s="24" t="s">
         <v>37</v>
       </c>
@@ -11524,7 +11530,7 @@
       <c r="DH32" s="8"/>
       <c r="DI32" s="8"/>
       <c r="DJ32" s="16"/>
-      <c r="DK32" s="35"/>
+      <c r="DK32" s="33"/>
       <c r="DL32" s="13"/>
       <c r="DM32" s="13"/>
       <c r="DN32" s="13"/>
@@ -11540,7 +11546,7 @@
       <c r="DX32" s="16"/>
     </row>
     <row r="33" spans="1:128" s="3" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="39"/>
+      <c r="A33" s="47"/>
       <c r="B33" s="22" t="s">
         <v>38</v>
       </c>
@@ -11672,7 +11678,7 @@
       <c r="DX33" s="7"/>
     </row>
     <row r="34" spans="1:128" s="3" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="40"/>
+      <c r="A34" s="48"/>
       <c r="B34" s="26" t="s">
         <v>39</v>
       </c>
@@ -11798,10 +11804,10 @@
       <c r="DR34" s="31"/>
       <c r="DS34" s="31"/>
       <c r="DT34" s="31"/>
-      <c r="DU34" s="36"/>
-      <c r="DV34" s="36"/>
-      <c r="DW34" s="36"/>
-      <c r="DX34" s="37"/>
+      <c r="DU34" s="34"/>
+      <c r="DV34" s="34"/>
+      <c r="DW34" s="34"/>
+      <c r="DX34" s="35"/>
     </row>
     <row r="35" spans="1:128" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="20"/>
@@ -12844,6 +12850,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A12:A23"/>
+    <mergeCell ref="A24:A34"/>
+    <mergeCell ref="BG2:BT4"/>
+    <mergeCell ref="BU2:CH4"/>
+    <mergeCell ref="CI2:CV4"/>
     <mergeCell ref="CW2:DJ4"/>
     <mergeCell ref="DK2:DX4"/>
     <mergeCell ref="A8:A11"/>
@@ -12853,11 +12864,6 @@
     <mergeCell ref="Q2:AD4"/>
     <mergeCell ref="AE2:AR4"/>
     <mergeCell ref="AS2:BF4"/>
-    <mergeCell ref="A12:A23"/>
-    <mergeCell ref="A24:A34"/>
-    <mergeCell ref="BG2:BT4"/>
-    <mergeCell ref="BU2:CH4"/>
-    <mergeCell ref="CI2:CV4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>